<commit_message>
Screenshots and sales report from the 30/30 todays-fixes run
Output of the e2eTodaysFixes suite against the current build: the nine
phase screenshots and the Sales Report it exported. Same nine files as
before, re-captured — the suite regenerates all of them every run.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/todays-fixes/sales-report.xlsx
+++ b/e2e-screenshots/todays-fixes/sales-report.xlsx
@@ -340,7 +340,7 @@
     <t>Carriage costed from</t>
   </si>
   <si>
-    <t>2026-08-05</t>
+    <t>2026-08-06</t>
   </si>
   <si>
     <t>Uncosted (pre-tracking) returns</t>
@@ -1155,7 +1155,7 @@
         <v>59</v>
       </c>
       <c r="C2" s="12">
-        <v>46179.5</v>
+        <v>46180.5</v>
       </c>
       <c r="D2" t="s">
         <v>121</v>
@@ -1178,7 +1178,7 @@
         <v>59</v>
       </c>
       <c r="C3" s="12">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="D3" t="s">
         <v>122</v>
@@ -1201,7 +1201,7 @@
         <v>59</v>
       </c>
       <c r="C4" s="12">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="D4" t="s">
         <v>122</v>
@@ -1224,7 +1224,7 @@
         <v>59</v>
       </c>
       <c r="C5" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="D5" s="9" t="s">
         <v>125</v>
@@ -1247,7 +1247,7 @@
         <v>59</v>
       </c>
       <c r="C6" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>125</v>
@@ -1370,7 +1370,7 @@
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="B2" s="9" t="s">
         <v>56</v>
@@ -1439,7 +1439,7 @@
         <v>59</v>
       </c>
       <c r="X2" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="Y2" s="9" t="s">
         <v>60</v>
@@ -1465,7 +1465,7 @@
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" s="12">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="B3" t="s">
         <v>64</v>
@@ -1545,7 +1545,7 @@
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="B4" s="9" t="s">
         <v>68</v>
@@ -1614,7 +1614,7 @@
         <v>59</v>
       </c>
       <c r="X4" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="Y4" s="9" t="s">
         <v>60</v>
@@ -1640,7 +1640,7 @@
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" s="12">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
@@ -1720,7 +1720,7 @@
     </row>
     <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" s="12">
-        <v>46211.5</v>
+        <v>46212.5</v>
       </c>
       <c r="B6" t="s">
         <v>72</v>
@@ -1800,7 +1800,7 @@
     </row>
     <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" s="12">
-        <v>46211.5</v>
+        <v>46212.5</v>
       </c>
       <c r="B7" t="s">
         <v>74</v>
@@ -1880,7 +1880,7 @@
     </row>
     <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" s="12">
-        <v>46211.5</v>
+        <v>46212.5</v>
       </c>
       <c r="B8" t="s">
         <v>76</v>
@@ -45368,7 +45368,7 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>57</v>
@@ -45386,7 +45386,7 @@
         <v>58</v>
       </c>
       <c r="G2" s="8">
-        <v>46239.5</v>
+        <v>46240.5</v>
       </c>
       <c r="H2" s="11">
         <v>610</v>

</xml_diff>

<commit_message>
Todays-fixes artefacts, re-captured after the GP correction
Same 30/30. The suite regenerates its fixtures and screenshots every run.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/e2e-screenshots/todays-fixes/sales-report.xlsx
+++ b/e2e-screenshots/todays-fixes/sales-report.xlsx
@@ -1424,7 +1424,7 @@
         <f>L2+N2+P2</f>
       </c>
       <c r="S2" s="11">
-        <f>I2-J2-K2-L2-M2-N2-O2-P2-Q2</f>
+        <v>0</v>
       </c>
       <c r="T2" s="11">
         <f>(S2-AB2)/G2*100</f>
@@ -1599,7 +1599,7 @@
         <f>L4+N4+P4</f>
       </c>
       <c r="S4" s="11">
-        <f>I4-J4-K4-L4-M4-N4-O4-P4-Q4</f>
+        <v>0</v>
       </c>
       <c r="T4" s="11">
         <f>(S4-AB4)/G4*100</f>

</xml_diff>